<commit_message>
Actualizar memoria (tablas 61 y 62 + texto) y Excel con agrupacion geometrica de vigas (d=342.6); coherencia memoria-Excel
</commit_message>
<xml_diff>
--- a/Proyectos/Diseno-Estructural/Reagrupacion-Geometrica-Vigas.xlsx
+++ b/Proyectos/Diseno-Estructural/Reagrupacion-Geometrica-Vigas.xlsx
@@ -93,14 +93,12 @@
     <col min="12" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
-    <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">REAGRUPACIÓN POR GEOMETRÍA (misma longitud + apoyos) — Diseño con la mayor solicitación del grupo · NSR-10 · sismo ÷ R=5</t>
+          <t xml:space="preserve">REAGRUPACIÓN POR GEOMETRÍA (misma longitud + apoyos) — Diseño con la mayor solicitación del grupo · NSR-10 · sismo ÷ R=5 · d=342.6 mm</t>
         </is>
       </c>
     </row>
@@ -157,30 +155,20 @@
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">As⁻ (mm²)</t>
+          <t xml:space="preserve">Ref. sup.</t>
         </is>
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ref. sup.</t>
+          <t xml:space="preserve">Ref. inf.</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">As⁺ (mm²)</t>
+          <t xml:space="preserve">φVc (kN)</t>
         </is>
       </c>
       <c r="N2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ref. inf.</t>
-        </is>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">φVc (kN)</t>
-        </is>
-      </c>
-      <c r="P2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Estribo #3</t>
         </is>
@@ -203,7 +191,7 @@
         </is>
       </c>
       <c r="D3" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E3" s="3">
         <v>2.5</v>
@@ -223,28 +211,22 @@
       <c r="J3" s="3">
         <v>1.9</v>
       </c>
-      <c r="K3" s="3">
-        <v>350</v>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº5</t>
+        </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2#5</t>
+          <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
       <c r="M3" s="3">
-        <v>350</v>
+        <v>69.3</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2#5</t>
-        </is>
-      </c>
-      <c r="O3" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -265,7 +247,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E4" s="3">
         <v>2.6</v>
@@ -285,28 +267,22 @@
       <c r="J4" s="3">
         <v>0.3</v>
       </c>
-      <c r="K4" s="3">
-        <v>350</v>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Nº5</t>
+        </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2#5</t>
+          <t xml:space="preserve">2 Nº5</t>
         </is>
       </c>
       <c r="M4" s="3">
-        <v>350</v>
+        <v>69.3</v>
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2#5</t>
-        </is>
-      </c>
-      <c r="O4" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -327,7 +303,7 @@
         </is>
       </c>
       <c r="D5" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E5" s="3">
         <v>2.65</v>
@@ -347,28 +323,22 @@
       <c r="J5" s="3">
         <v>0</v>
       </c>
-      <c r="K5" s="3">
-        <v>979</v>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 Nº5</t>
+        </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
+          <t xml:space="preserve">5 Nº5</t>
         </is>
       </c>
       <c r="M5" s="3">
-        <v>836</v>
+        <v>69.3</v>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
-        </is>
-      </c>
-      <c r="O5" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -389,7 +359,7 @@
         </is>
       </c>
       <c r="D6" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E6" s="3">
         <v>3.75</v>
@@ -409,28 +379,22 @@
       <c r="J6" s="3">
         <v>0</v>
       </c>
-      <c r="K6" s="3">
-        <v>864</v>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M6" s="3">
-        <v>721</v>
+        <v>69.3</v>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O6" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -451,7 +415,7 @@
         </is>
       </c>
       <c r="D7" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E7" s="3">
         <v>3.81</v>
@@ -471,28 +435,22 @@
       <c r="J7" s="3">
         <v>6.9</v>
       </c>
-      <c r="K7" s="3">
-        <v>935</v>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M7" s="3">
-        <v>648</v>
+        <v>69.3</v>
       </c>
       <c r="N7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O7" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -513,7 +471,7 @@
         </is>
       </c>
       <c r="D8" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E8" s="3">
         <v>3.85</v>
@@ -533,28 +491,22 @@
       <c r="J8" s="3">
         <v>0</v>
       </c>
-      <c r="K8" s="3">
-        <v>1004</v>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 Nº5</t>
+        </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M8" s="3">
-        <v>753</v>
+        <v>69.3</v>
       </c>
       <c r="N8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O8" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -575,7 +527,7 @@
         </is>
       </c>
       <c r="D9" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E9" s="3">
         <v>3.9</v>
@@ -595,28 +547,22 @@
       <c r="J9" s="3">
         <v>0</v>
       </c>
-      <c r="K9" s="3">
-        <v>1070</v>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6 Nº5</t>
+        </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M9" s="3">
-        <v>730</v>
+        <v>69.3</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O9" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -637,7 +583,7 @@
         </is>
       </c>
       <c r="D10" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E10" s="3">
         <v>4.0</v>
@@ -657,28 +603,22 @@
       <c r="J10" s="3">
         <v>0</v>
       </c>
-      <c r="K10" s="3">
-        <v>846</v>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M10" s="3">
-        <v>700</v>
+        <v>69.3</v>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O10" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -699,7 +639,7 @@
         </is>
       </c>
       <c r="D11" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E11" s="3">
         <v>5.1</v>
@@ -719,28 +659,22 @@
       <c r="J11" s="3">
         <v>0</v>
       </c>
-      <c r="K11" s="3">
-        <v>789</v>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M11" s="3">
-        <v>563</v>
+        <v>69.3</v>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O11" s="3">
-        <v>70.8</v>
-      </c>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -761,7 +695,7 @@
         </is>
       </c>
       <c r="D12" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E12" s="3">
         <v>1.5</v>
@@ -781,28 +715,22 @@
       <c r="J12" s="3">
         <v>25.7</v>
       </c>
-      <c r="K12" s="3">
-        <v>453</v>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M12" s="3">
-        <v>429</v>
+        <v>80.9</v>
       </c>
       <c r="N12" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O12" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P12" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -823,7 +751,7 @@
         </is>
       </c>
       <c r="D13" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E13" s="3">
         <v>2.5</v>
@@ -843,28 +771,22 @@
       <c r="J13" s="3">
         <v>0.6</v>
       </c>
-      <c r="K13" s="3">
-        <v>408</v>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M13" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O13" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -885,7 +807,7 @@
         </is>
       </c>
       <c r="D14" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E14" s="3">
         <v>2.6</v>
@@ -905,28 +827,22 @@
       <c r="J14" s="3">
         <v>6.4</v>
       </c>
-      <c r="K14" s="3">
-        <v>777</v>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
+          <t xml:space="preserve">4 Nº5</t>
         </is>
       </c>
       <c r="M14" s="3">
-        <v>691</v>
+        <v>80.9</v>
       </c>
       <c r="N14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
-        </is>
-      </c>
-      <c r="O14" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -947,7 +863,7 @@
         </is>
       </c>
       <c r="D15" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E15" s="3">
         <v>2.7</v>
@@ -967,28 +883,22 @@
       <c r="J15" s="3">
         <v>4.2</v>
       </c>
-      <c r="K15" s="3">
-        <v>643</v>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M15" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O15" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1009,7 +919,7 @@
         </is>
       </c>
       <c r="D16" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E16" s="3">
         <v>2.8</v>
@@ -1029,28 +939,22 @@
       <c r="J16" s="3">
         <v>4.0</v>
       </c>
-      <c r="K16" s="3">
-        <v>624</v>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M16" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N16" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O16" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1071,7 +975,7 @@
         </is>
       </c>
       <c r="D17" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E17" s="3">
         <v>2.95</v>
@@ -1091,28 +995,22 @@
       <c r="J17" s="3">
         <v>1.7</v>
       </c>
-      <c r="K17" s="3">
-        <v>437</v>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M17" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O17" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1031,7 @@
         </is>
       </c>
       <c r="D18" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E18" s="3">
         <v>3.3</v>
@@ -1153,28 +1051,22 @@
       <c r="J18" s="3">
         <v>1.1</v>
       </c>
-      <c r="K18" s="3">
-        <v>408</v>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M18" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N18" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O18" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1087,7 @@
         </is>
       </c>
       <c r="D19" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E19" s="3">
         <v>3.65</v>
@@ -1215,28 +1107,22 @@
       <c r="J19" s="3">
         <v>6.0</v>
       </c>
-      <c r="K19" s="3">
-        <v>408</v>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M19" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O19" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1143,7 @@
         </is>
       </c>
       <c r="D20" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E20" s="3">
         <v>4.0</v>
@@ -1277,28 +1163,22 @@
       <c r="J20" s="3">
         <v>5.5</v>
       </c>
-      <c r="K20" s="3">
-        <v>512</v>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 Nº5</t>
+        </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M20" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O20" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1199,7 @@
         </is>
       </c>
       <c r="D21" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E21" s="3">
         <v>4.18</v>
@@ -1339,28 +1219,22 @@
       <c r="J21" s="3">
         <v>0.8</v>
       </c>
-      <c r="K21" s="3">
-        <v>617</v>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 Nº5</t>
+        </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M21" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O21" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1255,7 @@
         </is>
       </c>
       <c r="D22" s="3">
-        <v>350</v>
+        <v>342.6</v>
       </c>
       <c r="E22" s="3">
         <v>5.5</v>
@@ -1401,28 +1275,22 @@
       <c r="J22" s="3">
         <v>0.0</v>
       </c>
-      <c r="K22" s="3">
-        <v>835</v>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Nº5</t>
+        </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5#5</t>
+          <t xml:space="preserve">3 Nº5</t>
         </is>
       </c>
       <c r="M22" s="3">
-        <v>408</v>
+        <v>80.9</v>
       </c>
       <c r="N22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3#5</t>
-        </is>
-      </c>
-      <c r="O22" s="3">
-        <v>82.6</v>
-      </c>
-      <c r="P22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">@88mm(2h)/@175mm</t>
+          <t xml:space="preserve">@86mm(2h)/@171mm</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1308,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">METODOLOGÍA DE AGRUPACIÓN (indicación del Ing. Sergio Ladino)</t>
+          <t xml:space="preserve">METODOLOGÍA (indicación Ing. Sergio Ladino)</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1323,7 @@
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agrupar vigas con la MISMA longitud y las MISMAS condiciones de apoyo; diseñar y despiezar con la MAYOR solicitación del grupo.</t>
+          <t xml:space="preserve">Agrupar vigas con MISMA longitud y MISMAS condiciones de apoyo; diseñar con la MAYOR solicitación del grupo.</t>
         </is>
       </c>
     </row>
@@ -1470,31 +1338,31 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP2000 - Element Forces-Frames (COMB1..10) + Frame Section Assignments.</t>
+          <t xml:space="preserve">SAP2000 (Element Forces + Frame Section Assignments). Longitud = máx Station. d=342.6 mm (rec.40+estribo#3+½#5).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longitud:</t>
+          <t xml:space="preserve">Secciones:</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">máxima 'Station' de cada frame.</t>
+          <t xml:space="preserve">VC40x30 carga (b=300). VR40x35 rigidez (b=350). h=400. f'c=28 MPa, fy=420 MPa.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secciones:</t>
+          <t xml:space="preserve">Sismo:</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">VC40x30 = vigas de carga (b=300,h=400). VR40x35 = vigas de rigidez/riostras (b=350,h=400).</t>
+          <t xml:space="preserve">Fx,Fy elásticas (Vs=0.45W). Diseño con E÷R=5 estación por estación. Derivas con fuerza sin reducir.</t>
         </is>
       </c>
     </row>
@@ -1504,77 +1372,12 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sismo:</t>
+          <t xml:space="preserve">Viguetas:</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fx,Fy del modelo son ELÁSTICAS (Vs=0.45W, sin R). Para diseño se reduce E÷R=5, estación por estación:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="0"/>
-      <c r="B10" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gravedad=(COMB3+COMB4)/2 ; Sismo=(COMB3-COMB4)/2 ; Diseño=Gravedad+Sismo/R. Derivas: con fuerza sin reducir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="0"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Materiales:</t>
-        </is>
-      </c>
-      <c r="B12" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">f'c=28 MPa; fy=420 MPa; φflexión=0.90; φcortante=0.75. As,min=1.4·b·d/fy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Estribos:</t>
-        </is>
-      </c>
-      <c r="B13" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#3 (2 ramas). Confinamiento DMO 2h: s≤mín(d/4,6dbL,150). Resto: s≤d/2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="0"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Viguetas:</t>
-        </is>
-      </c>
-      <c r="B15" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No están en SAP (nervios de losa). Se agrupan por LUZ (entrepiso/cubierta) = cumple el criterio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOTA:</t>
-        </is>
-      </c>
-      <c r="B17" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Esta agrupación reemplaza la anterior por rangos de momento. Los momentos de diseño quedan menores y realistas (máx VC≈129, VR≈104 kN·m).</t>
+          <t xml:space="preserve">Agrupadas por luz (entrepiso/cubierta) = cumplen el criterio.</t>
         </is>
       </c>
     </row>

</xml_diff>